<commit_message>
Refresh generated reports after validation
</commit_message>
<xml_diff>
--- a/reports/REPORTE_VENTAS.xlsx
+++ b/reports/REPORTE_VENTAS.xlsx
@@ -22,13 +22,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +42,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,12 +50,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -422,102 +434,102 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Actividades</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Almacén</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Empresa</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Equipo de ventas</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Estado de la factura</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Etiquetas</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Excepción principal</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Fecha de creación</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Fecha de entrega</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Fecha esperada</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Impuestos</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Referencia de la orden</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Referencia del cliente</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Términos de pago</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Vencimiento</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Vendedor</t>
         </is>
@@ -6590,29 +6602,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Monto Total</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Promedio</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>ROBERTO PICCA E HIJOS S.A.S.</t>
         </is>
@@ -6628,7 +6640,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>BENITEZ MATIAS</t>
         </is>
@@ -6644,7 +6656,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>INFINITY SAS</t>
         </is>
@@ -6660,7 +6672,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>GUETE HECTOR DANIEL</t>
         </is>
@@ -6676,7 +6688,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>BURLOTTI FEDERICO VICTOR</t>
         </is>
@@ -6692,7 +6704,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>MARTIN DANIEL JOSE</t>
         </is>
@@ -6708,7 +6720,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>GUTIERREZ LUCAS DAVID</t>
         </is>
@@ -6724,7 +6736,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>S&amp;L EQUIPAMIENTOS S.A.</t>
         </is>
@@ -6740,7 +6752,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>SUEÑO LINDO S. A. S.</t>
         </is>
@@ -6756,7 +6768,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>AVALOS LOURDES SOLEDAD</t>
         </is>
@@ -6772,7 +6784,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>KRAAP WALTER</t>
         </is>
@@ -6788,7 +6800,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>LA FE SRL</t>
         </is>
@@ -6804,7 +6816,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>PARDO S.A.</t>
         </is>
@@ -6820,7 +6832,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>FERNANDEZ WALTER RAUL</t>
         </is>
@@ -6836,7 +6848,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>FARA LUIS</t>
         </is>
@@ -6852,7 +6864,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>CROCE SILVIA ESTHER</t>
         </is>
@@ -6868,7 +6880,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>MARIANI ORNELLA</t>
         </is>
@@ -6884,7 +6896,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>ANGEL MARIA ANTONIETA</t>
         </is>
@@ -6900,7 +6912,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>PONS RODRIGO</t>
         </is>
@@ -6916,7 +6928,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>DIST. CONFORTAN S.A.C.I.</t>
         </is>
@@ -6932,7 +6944,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>GRIFFA ANDRES</t>
         </is>
@@ -6948,7 +6960,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>MARTINUZZI RAUL OMAR</t>
         </is>
@@ -6964,7 +6976,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>FERREYRA ELOY JOSE</t>
         </is>
@@ -6980,7 +6992,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="1" t="inlineStr">
         <is>
           <t>CHAUD ROBERTO ARIEL</t>
         </is>
@@ -6996,7 +7008,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>MALDONADO MARCELA FABIANA</t>
         </is>
@@ -7012,7 +7024,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>BORIGLIO FRANCO</t>
         </is>
@@ -7028,7 +7040,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="1" t="inlineStr">
         <is>
           <t>CIARLANTINI MYRIAM DEL LUJAN</t>
         </is>
@@ -7044,7 +7056,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t>LEFERP SRL</t>
         </is>
@@ -7060,7 +7072,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="1" t="inlineStr">
         <is>
           <t>NACUSI SERGIO FERNANDO</t>
         </is>
@@ -7076,7 +7088,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>MARTINEZ RAUL</t>
         </is>
@@ -7092,7 +7104,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>ERXILAPE JUAN CARLOS</t>
         </is>
@@ -7108,7 +7120,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="1" t="inlineStr">
         <is>
           <t>ABDO LUCIANA BELEN</t>
         </is>
@@ -7124,7 +7136,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="1" t="inlineStr">
         <is>
           <t>NACUSI EDUARDO ERNESTO</t>
         </is>
@@ -7140,7 +7152,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="1" t="inlineStr">
         <is>
           <t>GRIFFA ARIEL</t>
         </is>
@@ -7156,7 +7168,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="1" t="inlineStr">
         <is>
           <t>EGGSTEIN CLAUDIO</t>
         </is>
@@ -7172,7 +7184,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="1" t="inlineStr">
         <is>
           <t>VITOBALDI LUCIA ANDREA</t>
         </is>
@@ -7188,7 +7200,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="1" t="inlineStr">
         <is>
           <t>MUHN SUNILDA ADRIANA</t>
         </is>
@@ -7204,7 +7216,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="1" t="inlineStr">
         <is>
           <t>J.T.M.M CONCEPTION S. A.</t>
         </is>
@@ -7220,7 +7232,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="1" t="inlineStr">
         <is>
           <t>ARMAR S.R.L</t>
         </is>
@@ -7236,7 +7248,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="1" t="inlineStr">
         <is>
           <t>LA PAMPA HOGAR S.H</t>
         </is>
@@ -7252,7 +7264,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="1" t="inlineStr">
         <is>
           <t>LUX HOGAR S.A.</t>
         </is>
@@ -7268,7 +7280,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="1" t="inlineStr">
         <is>
           <t>REISENAUER MARIA SOLEDAD</t>
         </is>
@@ -7284,7 +7296,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="1" t="inlineStr">
         <is>
           <t>MUEBLES MALPASSI Y OBERTI OBERTI SRL</t>
         </is>
@@ -7300,7 +7312,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="1" t="inlineStr">
         <is>
           <t>DUCHOSAL LUZ ROXANA MARICEL</t>
         </is>
@@ -7316,7 +7328,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="1" t="inlineStr">
         <is>
           <t>BONALDI SRL</t>
         </is>
@@ -7332,7 +7344,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="1" t="inlineStr">
         <is>
           <t>PUIGRREDON SEBASTIAN</t>
         </is>
@@ -7348,7 +7360,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="1" t="inlineStr">
         <is>
           <t>LUDUEÑA GUSTAVO</t>
         </is>
@@ -7364,7 +7376,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="1" t="inlineStr">
         <is>
           <t>CIANI JORDAN SANTIAGO</t>
         </is>
@@ -7380,7 +7392,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="1" t="inlineStr">
         <is>
           <t>COMPAGNUCCI MARIEL</t>
         </is>
@@ -7396,7 +7408,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="1" t="inlineStr">
         <is>
           <t>GERBALDO REFRIGERACION S.R.L.</t>
         </is>
@@ -7412,7 +7424,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="1" t="inlineStr">
         <is>
           <t>TALLERES CHICAGO S.A.</t>
         </is>
@@ -7428,7 +7440,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="1" t="inlineStr">
         <is>
           <t>BUCALA GUSTAVO R. Y BUCALA HORACIO S.H.</t>
         </is>
@@ -7444,7 +7456,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="1" t="inlineStr">
         <is>
           <t>AIMAR CARLOS NAHUEL</t>
         </is>
@@ -7460,7 +7472,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="1" t="inlineStr">
         <is>
           <t>JB AMOBLAMIENTOS S.A.S.</t>
         </is>
@@ -7476,7 +7488,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="1" t="inlineStr">
         <is>
           <t>RADIO PEYBO TV SACIFI</t>
         </is>
@@ -7492,7 +7504,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="1" t="inlineStr">
         <is>
           <t>GAR-BON S.A.S</t>
         </is>
@@ -7508,7 +7520,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="1" t="inlineStr">
         <is>
           <t>SANCHEZ PABLO ANDRES</t>
         </is>
@@ -7524,7 +7536,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="1" t="inlineStr">
         <is>
           <t>CALDO ALEJANDRO FABIAN</t>
         </is>
@@ -7540,7 +7552,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="1" t="inlineStr">
         <is>
           <t>PONCE DE LEON JUAN CRUZ</t>
         </is>
@@ -7556,7 +7568,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="1" t="inlineStr">
         <is>
           <t>SCHMIDT Y BAYER  S.R.L.</t>
         </is>
@@ -7572,7 +7584,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="1" t="inlineStr">
         <is>
           <t>BONNIN MARCELO</t>
         </is>
@@ -7588,7 +7600,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="1" t="inlineStr">
         <is>
           <t>MASHALLA S.A.S</t>
         </is>
@@ -7604,7 +7616,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="1" t="inlineStr">
         <is>
           <t>LA CASA DEL TAPICERO S.R.L.</t>
         </is>
@@ -7620,7 +7632,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="1" t="inlineStr">
         <is>
           <t>BERTOLA EMILIANO JESUS</t>
         </is>
@@ -7636,7 +7648,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="1" t="inlineStr">
         <is>
           <t>KRESS S.A.</t>
         </is>
@@ -7652,7 +7664,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="1" t="inlineStr">
         <is>
           <t>SANCHEZ MUEBLES PERGAMINO S.R.L</t>
         </is>
@@ -7668,7 +7680,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" s="1" t="inlineStr">
         <is>
           <t>FIERRO CAROLINA</t>
         </is>
@@ -7684,7 +7696,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="1" t="inlineStr">
         <is>
           <t>MADERSORO SA</t>
         </is>
@@ -7700,7 +7712,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" s="1" t="inlineStr">
         <is>
           <t>MICHELOTTI DARIO</t>
         </is>
@@ -7716,7 +7728,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
+      <c r="A71" s="1" t="inlineStr">
         <is>
           <t>RAYCES S.R.L.</t>
         </is>
@@ -7732,7 +7744,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
+      <c r="A72" s="1" t="inlineStr">
         <is>
           <t>RICCI MIGUEL ANGEL</t>
         </is>
@@ -7762,34 +7774,34 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Vendedor</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Monto Total</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Órdenes</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Promedio</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Clientes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Bermudez Bruno</t>
         </is>
@@ -7808,7 +7820,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Caamaño Andrés</t>
         </is>
@@ -7827,7 +7839,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Campo Eduardo - Victor Orpianessi</t>
         </is>
@@ -7846,7 +7858,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Civile Tomas</t>
         </is>
@@ -7865,7 +7877,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Giagante Federico</t>
         </is>
@@ -7884,7 +7896,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>Horacio Lopez</t>
         </is>
@@ -7903,7 +7915,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>Maggi Mauro</t>
         </is>
@@ -7922,7 +7934,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>Miranda Mario</t>
         </is>
@@ -7955,12 +7967,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
@@ -8065,19 +8077,19 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Orden de venta</t>
         </is>
@@ -8087,7 +8099,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Cotización</t>
         </is>
@@ -8097,7 +8109,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Pendiente de aprobación</t>
         </is>
@@ -8121,19 +8133,19 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Términos de pago</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>30, 60, 90 y 120 días</t>
         </is>
@@ -8143,7 +8155,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Presupuesto</t>
         </is>
@@ -8153,7 +8165,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>30, 60, 90, 120, y 150 días</t>
         </is>
@@ -8163,7 +8175,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Pago anticipado</t>
         </is>
@@ -8173,7 +8185,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>30 días</t>
         </is>
@@ -8183,7 +8195,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>20 días</t>
         </is>
@@ -8193,7 +8205,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>30, 60, 90 días</t>
         </is>

</xml_diff>